<commit_message>
Update Excel files in the Analys directory with new data and corrections
- Modified Programkurser olankade.xlsx
- Updated Samstämighet svenska och engelska.xlsx
- Corrected Stavfel och språkbruk.xlsx
- Revised Övrigt.xlsx
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/01 IIT/Analys/Programkurser olankade.xlsx
+++ b/vault-dalarna-university/01 IIT/Analys/Programkurser olankade.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Programkurser olankade" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olankade'!$A$1:$E$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Programkurser olankade'!$A$1:$E$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -563,12 +563,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Kurs finns aktivt men scrapern länkade inte</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>`System- och verksamhetsutveckling` (7,5hp); rad: - System- och verksamhetsutveckling, 7,5hp</t>
+          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5hp</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -644,12 +644,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Kurs finns aktivt men scrapern länkade inte</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>`System- och verksamhetsutveckling` (7,5 hp); rad: - System- och verksamhetsutveckling, 7,5 hp</t>
+          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5 hp</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -661,7 +661,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>KGDWG</t>
+          <t>DSVPG</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -671,24 +671,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Kurs finns aktivt men scrapern länkade inte</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>`System- och verksamhetsutveckling` (7,5 hp); rad: - System- och verksamhetsutveckling, 7,5 hp</t>
+          <t>Programtext `Webbaserade geografiska informationssystem` ≠ kursplanens namn `Webbaserade geografiska informationssystem (GIS)` (kurskod `GIK2JX`); rad: - [[GIK2JX|Webbaserade geografiska informationssystem]], 7,5 hp</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KGDWG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=DSVPG</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TATPG</t>
+          <t>KGDWG</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -698,17 +698,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>`Forskningsmetodik för ingenjörer` (7,5hp); rad: - Forskningsmetodik för ingenjörer, 7,5hp</t>
+          <t>Programtext `System- och verksamhetsutveckling` ≠ kursplanens namn `System och verksamhetsutveckling` (kurskod `GIK2XZ`); rad: - [[GIK2XZ|System- och verksamhetsutveckling]], 7,5 hp</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=KGDWG</t>
         </is>
       </c>
     </row>
@@ -730,7 +730,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>`Examensarbete i assisterande teknik med inriktning mot maskinteknik` (15 hp); rad: - Examensarbete i assisterande teknik med inriktning mot maskinteknik, 15 hp</t>
+          <t>`Forskningsmetodik för ingenjörer` (7,5hp); rad: - Forskningsmetodik för ingenjörer, 7,5hp</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden i praktiken` (7,5 hp); rad: - Finita elementmetoden i praktiken, 7,5 hp</t>
+          <t>`Examensarbete i assisterande teknik med inriktning mot maskinteknik` (15 hp); rad: - Examensarbete i assisterande teknik med inriktning mot maskinteknik, 15 hp</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -769,7 +769,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>TBYSG</t>
+          <t>TATPG</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -784,19 +784,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp); rad: - Fysisk planering III – genomförande och planeringsjuridik, 7,5 hp</t>
+          <t>`Finita elementmetoden i praktiken` (7,5 hp); rad: - Finita elementmetoden i praktiken, 7,5 hp</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TATPG</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TMSSA</t>
+          <t>TBTCG</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -806,24 +806,24 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Kursraden ser avbruten/feltrycklig ut</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>`Solenergiteknikpraktik (7,5 eller` (15 hp); rad: - Solenergiteknikpraktik (7,5 eller, 15 hp</t>
+          <t>Programtext `Husbyggnadsprojekt I – Små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – Små byggnader och bostadsområden]], 15 hp</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TPOKG</t>
+          <t>TBTCG</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -833,24 +833,24 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
+          <t>Programtext `Husbyggnadsprojekt III – Byggkonstruktionsprojekt` ≠ kursplanens namn `Husbyggnadsprojekt III - Byggkonstruktionsprojekt` (kurskod `GBY3AX`); rad: - [[GBY3AX|Husbyggnadsprojekt III – Byggkonstruktionsprojekt]], 7,5 hp</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTCG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TBTFG</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -860,24 +860,24 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
+          <t>Programtext `Husbyggnadsprojekt I – små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – små byggnader och bostadsområden]], 15 hp</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBTFG</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TBYSG</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -892,19 +892,19 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
+          <t>`Fysisk planering III – genomförande och planeringsjuridik` (7,5 hp); rad: - Fysisk planering III – genomförande och planeringsjuridik, 7,5 hp</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TBYSG</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -914,24 +914,24 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
+          <t>Programtext `Husbyggnadsprojekt I – små byggnader och bostadsområden` ≠ kursplanens namn `Husbyggnadsprojekt I - Små byggnader och bostadsområden` (kurskod `GBY2J2`); rad: - [[GBY2J2|Husbyggnadsprojekt I – små byggnader och bostadsområden]], 15 hp</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TBYSG</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TEKHG</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -941,24 +941,24 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
+          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>TPTAG</t>
+          <t>TEKHG</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -968,49 +968,427 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bullet beskriver val mellan flera kurser</t>
+          <t>Programtext avviker från kursplanens namn</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>`CAM / CNC` (7,5 hp); rad: - CAM / CNC, 7,5 hp</t>
+          <t>Programtext `Industriell ekonomi – organisation och ledarskap` ≠ kursplanens namn `Industriell ekonomi - organisation och ledarskap` (kurskod `GIE26M`); rad: - [[GIE26M|Industriell ekonomi – organisation och ledarskap]], 7,5 hp</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
+          <t>TEKHG</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Programtext `Industriell ekonomi – underhåll och kvalitet` ≠ kursplanens namn `Industriell ekonomi - underhåll och kvalitet` (kurskod `GIE26N`); rad: - [[GIE26N|Industriell ekonomi – underhåll och kvalitet]], 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TEKHG</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>THIHG</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Programtext `Industriell ekonomi – grundläggande kurs` ≠ kursplanens namn `Industriell ekonomi - grundläggande kurs` (kurskod `GIE26P`); rad: - [[GIE26P|Industriell ekonomi – grundläggande kurs]], 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>THIHG</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Programtext `Utvecklingsprojekt, tillverkning av en solfångare` ≠ kursplanens namn `Utvecklingsprojekt, tillverkning av en solfångare` (kurskod `GEG2JP`); rad: - [[GEG2JP|Utvecklingsprojekt, tillverkning av en solfångare]], 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=THIHG</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>TMIEA</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Programtext `Byggnaders energiprestanda – simulering och analys` ≠ kursplanens namn `Byggnaders energiprestanda - simulering och analys` (kurskod `ABY22W`); rad: - [[ABY22W|Byggnaders energiprestanda – simulering och analys]], 5.0 hp</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMIEA</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>TMSSA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Kursraden ser avbruten/feltrycklig ut</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>`Solenergiteknikpraktik (7,5 eller` (15 hp); rad: - Solenergiteknikpraktik (7,5 eller, 15 hp</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>TMSSA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Programtext `Projektkurs 1 – dataanalys för solenergisystem` ≠ kursplanens namn `Projektkurs 1 - dataanalys för solenergisystem` (kurskod `AEG2AK`); rad: - [[AEG2AK|Projektkurs 1 – dataanalys för solenergisystem]], 5 hp</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>TMSSA</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Programtext `Projektkurs 2 – mätsystem` ≠ kursplanens namn `Projektkurs 2 - mätsystem` (kurskod `AEG2AU`); rad: - [[AEG2AU|Projektkurs 2 – mätsystem]], 5 hp</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>TMSSA</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Programtext avviker från kursplanens namn</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Programtext `Projektkurs 3 – grupprojekt och kommunikation` ≠ kursplanens namn `Projektkurs 3 - grupprojekt och kommunikation` (kurskod `AEG2B5`); rad: - [[AEG2B5|Projektkurs 3 – grupprojekt och kommunikation]], 5 hp</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TMSSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>TPOKG</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>`Finita elementmetoden` (7,5hp); rad: - Finita elementmetoden, 7,5hp</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPOKG</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>TPTAG</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>`3D CAD grundkurs` (7,5 hp); rad: - 3D CAD grundkurs, 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>TPTAG</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>`Additiv tillverkning` (7,5 hp); rad: - Additiv tillverkning, 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>TPTAG</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>`Examensarbete för högskoleexamen inom maskinteknik` (7,5 hp); rad: - Examensarbete för högskoleexamen inom maskinteknik, 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>TPTAG</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Kursnamnet finns varken aktivt eller nedlagt</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>`Underhåll och kvalitet` (7,5 hp); rad: - Underhåll och kvalitet, 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>TPTAG</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Bullet beskriver val mellan flera kurser</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>`CAM / CNC` (7,5 hp); rad: - CAM / CNC, 7,5 hp</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TPTAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
           <t>TSETA</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Utbildningsplan</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Utbildningsplan</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
         <is>
           <t>Kursnamnet finns varken aktivt eller nedlagt</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>`Design av PV hybrid system` (7,5 hp); rad: - Design av PV hybrid system, 7,5 hp</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="E35" s="2" t="inlineStr">
         <is>
           <t>https://www.du.se/sv/utbildning/Program/utbildningsplan/?code=TSETA</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E21"/>
+  <autoFilter ref="A1:E35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId2"/>
@@ -1052,6 +1430,34 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E20" r:id="rId38"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId39"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId68"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>